<commit_message>
fixed a excel formula in asu definition that is not compatible with libreoffice
</commit_message>
<xml_diff>
--- a/models/demo-spatial/demo-spatial.xlsx
+++ b/models/demo-spatial/demo-spatial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-models/demo-spatial/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27FD5776-0A36-9444-B07E-D704D7BA8079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892549BD-AA6A-D645-943D-CECD0E22F4CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="180" yWindow="600" windowWidth="40560" windowHeight="26860" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,28 +58,6 @@
 </comments>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="140">
   <si>
@@ -507,7 +485,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -532,6 +510,11 @@
       <color theme="0"/>
       <name val="HelveticaNeue"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="HelveticaNeue"/>
     </font>
   </fonts>
   <fills count="4">
@@ -566,13 +549,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1452,8 +1436,7 @@
       <c r="B3" t="s">
         <v>50</v>
       </c>
-      <c r="C3" cm="1">
-        <f t="array" ref="C3">SUMPRODUCT(CODE(MID(D3, _xlfn.SEQUENCE(LEN(D3)), 1)), 31^(LEN(D3)-_xlfn.SEQUENCE(LEN(D3))))</f>
+      <c r="C3">
         <v>2113</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1467,8 +1450,7 @@
       <c r="B4" t="s">
         <v>50</v>
       </c>
-      <c r="C4" cm="1">
-        <f t="array" ref="C4">SUMPRODUCT(CODE(MID(D4, _xlfn.SEQUENCE(LEN(D4)), 1)), 31^(LEN(D4)-_xlfn.SEQUENCE(LEN(D4))))</f>
+      <c r="C4">
         <v>2081</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1482,8 +1464,7 @@
       <c r="B5" t="s">
         <v>50</v>
       </c>
-      <c r="C5" cm="1">
-        <f t="array" ref="C5">SUMPRODUCT(CODE(MID(D5, _xlfn.SEQUENCE(LEN(D5)), 1)), 31^(LEN(D5)-_xlfn.SEQUENCE(LEN(D5))))</f>
+      <c r="C5">
         <v>2762</v>
       </c>
       <c r="D5" s="5" t="s">
@@ -1787,7 +1768,7 @@
       <c r="D41" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" s="6" t="s">
         <v>22</v>
       </c>
       <c r="F41" s="1" t="s">

</xml_diff>